<commit_message>
Atualiza historico e state 2026-09-14 18:18 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,96 +485,96 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-11T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-10T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração de Membros do Conselho de Administração</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-09T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -589,64 +589,64 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-08T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -658,37 +658,37 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
         </is>
       </c>
     </row>
@@ -700,37 +700,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -742,133 +742,133 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-08-24T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -883,44 +883,44 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-18T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -952,17 +952,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -994,49 +994,49 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1056,39 +1056,39 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1098,39 +1098,39 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1140,39 +1140,39 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1204,37 +1204,37 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1246,17 +1246,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1271,12 +1271,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1288,37 +1288,37 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1345,86 +1345,86 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1434,71 +1434,71 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1513,34 +1513,34 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1555,64 +1555,64 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1639,160 +1639,160 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1817,118 +1817,118 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1943,34 +1943,34 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1980,71 +1980,71 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2069,34 +2069,34 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2106,29 +2106,29 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2143,34 +2143,34 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2185,34 +2185,34 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2227,34 +2227,34 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2274,249 +2274,249 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2531,24 +2531,24 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2568,123 +2568,123 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2694,59 +2694,59 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2758,17 +2758,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2783,12 +2783,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2820,17 +2820,17 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2857,22 +2857,22 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2899,22 +2899,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2941,22 +2941,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2968,37 +2968,37 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3030,29 +3030,29 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3067,34 +3067,34 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3109,111 +3109,279 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
-        </is>
-      </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="H70" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H66"/>
+  <autoFilter ref="A1:H70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-15 17:26 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1125,12 +1125,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1167,12 +1167,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1881,32 +1881,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2637,32 +2637,32 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2815,22 +2815,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2867,12 +2867,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2899,22 +2899,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2931,12 +2931,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2951,12 +2951,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2983,22 +2983,22 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3015,32 +3015,32 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3067,22 +3067,22 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3109,22 +3109,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-16 17:25 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1125,12 +1125,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1167,12 +1167,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1881,32 +1881,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2637,32 +2637,32 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2815,22 +2815,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2857,22 +2857,22 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2899,22 +2899,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2931,32 +2931,32 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2973,12 +2973,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2993,12 +2993,12 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3025,22 +3025,22 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3077,12 +3077,12 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3109,22 +3109,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-17 17:25 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1125,12 +1125,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1167,12 +1167,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1881,32 +1881,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2637,32 +2637,32 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2805,12 +2805,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2825,12 +2825,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2857,22 +2857,22 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2909,12 +2909,12 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2941,22 +2941,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2973,32 +2973,32 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3025,22 +3025,22 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3067,22 +3067,22 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3109,22 +3109,22 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-18 16:53 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1125,12 +1125,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1167,12 +1167,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1881,32 +1881,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2637,32 +2637,32 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2805,32 +2805,32 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2857,22 +2857,22 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2899,22 +2899,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2941,22 +2941,22 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2983,22 +2983,22 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3035,12 +3035,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3067,22 +3067,22 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3099,12 +3099,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -3119,12 +3119,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-19 16:11 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -1125,12 +1125,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1145,12 +1145,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1167,12 +1167,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1187,12 +1187,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1881,32 +1881,32 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1923,32 +1923,32 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2595,32 +2595,32 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2637,32 +2637,32 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2815,22 +2815,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2847,12 +2847,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2867,12 +2867,12 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2899,22 +2899,22 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2951,12 +2951,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2983,22 +2983,22 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3025,22 +3025,22 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3067,22 +3067,22 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3099,32 +3099,32 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-21 18:25 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,64 +485,64 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-11T00:00:00</t>
+          <t>2026-09-18T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-10T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -557,66 +557,66 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Alteração de Membros do Conselho de Administração</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-09T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-08T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -631,86 +631,86 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -725,34 +725,34 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -762,39 +762,39 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -804,71 +804,71 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -883,44 +883,44 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -930,123 +930,123 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-24T00:00:00</t>
+          <t>2026-09-15T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
+          <t>Reenquadramento da cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-11T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-10T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1061,34 +1061,34 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Alteração de Membros do Conselho de Administração</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-18T00:00:00</t>
+          <t>2026-09-09T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1098,29 +1098,29 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-09-08T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1140,197 +1140,197 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1345,34 +1345,34 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1387,34 +1387,34 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1429,76 +1429,76 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1528,29 +1528,29 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1565,34 +1565,34 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1602,197 +1602,197 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1817,34 +1817,34 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1854,29 +1854,29 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1891,34 +1891,34 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1933,44 +1933,44 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1985,24 +1985,24 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2017,44 +2017,44 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2069,34 +2069,34 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2106,49 +2106,49 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2158,81 +2158,81 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2242,187 +2242,187 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2442,39 +2442,39 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -2484,29 +2484,29 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2521,44 +2521,44 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2568,113 +2568,113 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2699,108 +2699,108 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2815,76 +2815,76 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2909,24 +2909,24 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2941,86 +2941,86 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3035,34 +3035,34 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3072,123 +3072,123 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3203,34 +3203,34 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3240,81 +3240,81 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -3329,59 +3329,563 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado - 1T26</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Assembleia</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultados 1T26</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Aviso aos Acionistas</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F70" t="inlineStr">
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G82" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="H82" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H70"/>
+  <autoFilter ref="A1:H82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-22 17:29 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -547,22 +547,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -594,17 +594,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -636,17 +636,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -673,22 +673,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -725,12 +725,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -762,17 +762,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1335,32 +1335,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2195,12 +2195,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3319,22 +3319,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3351,12 +3351,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3403,22 +3403,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3455,12 +3455,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3561,12 +3561,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3581,12 +3581,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-23 17:39 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -557,12 +557,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -594,17 +594,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -636,17 +636,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -673,22 +673,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -715,22 +715,22 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -762,17 +762,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
@@ -1335,32 +1335,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2195,12 +2195,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3319,22 +3319,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3351,12 +3351,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3403,22 +3403,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3455,12 +3455,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3561,12 +3561,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3581,12 +3581,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-24 17:42 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -547,22 +547,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -594,17 +594,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -636,17 +636,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -683,12 +683,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -715,22 +715,22 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -762,17 +762,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1335,32 +1335,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2195,12 +2195,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3319,22 +3319,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3351,12 +3351,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3403,22 +3403,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3455,12 +3455,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3561,12 +3561,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3581,12 +3581,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-25 17:43 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -547,22 +547,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -594,17 +594,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -636,17 +636,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -673,22 +673,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -725,12 +725,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -762,17 +762,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
@@ -1335,32 +1335,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2195,12 +2195,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3319,22 +3319,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3351,12 +3351,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3403,22 +3403,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3455,12 +3455,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3561,12 +3561,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3581,12 +3581,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-26 16:51 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -557,12 +557,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -594,17 +594,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -636,17 +636,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -673,22 +673,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -715,22 +715,22 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -762,17 +762,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1293,32 +1293,32 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1335,32 +1335,32 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2195,12 +2195,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3319,22 +3319,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Convocação AGE</t>
-        </is>
-      </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3351,12 +3351,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3371,12 +3371,12 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3403,22 +3403,22 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3455,12 +3455,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3561,12 +3561,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -3581,12 +3581,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-27 17:23 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H82"/>
+  <dimension ref="A1:H84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,12 +485,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-18T00:00:00</t>
+          <t>2026-09-22T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -520,49 +520,49 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-21T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-18T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -589,22 +589,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -683,12 +683,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -715,22 +715,22 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -762,17 +762,17 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -851,12 +851,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -883,22 +883,22 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -915,12 +915,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Publicação de Editais de Alienação de Imóveis</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -952,121 +952,121 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-15T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Reenquadramento da cotação das ações da Companhia</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-11T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-10T00:00:00</t>
+          <t>2026-09-15T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Alteração de Membros do Conselho de Administração</t>
+          <t>Reenquadramento da cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1078,37 +1078,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-09T00:00:00</t>
+          <t>2026-09-11T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
+          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1120,17 +1120,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-08T00:00:00</t>
+          <t>2026-09-10T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1140,29 +1140,29 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Alteração de Membros do Conselho de Administração</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-09T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1177,64 +1177,64 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-08T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1251,32 +1251,32 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1313,12 +1313,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
         </is>
       </c>
     </row>
@@ -1372,37 +1372,37 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1414,22 +1414,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1439,96 +1439,96 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-24T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
+          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1540,17 +1540,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1560,17 +1560,17 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1582,37 +1582,37 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-18T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1666,17 +1666,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1686,39 +1686,39 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1733,34 +1733,34 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1770,17 +1770,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1792,17 +1792,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1812,17 +1812,17 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1834,17 +1834,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1854,17 +1854,17 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1876,37 +1876,37 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1918,37 +1918,37 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1960,37 +1960,37 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2002,59 +2002,59 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2069,66 +2069,66 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2143,64 +2143,64 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2279,12 +2279,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2311,128 +2311,128 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2442,123 +2442,123 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2573,12 +2573,12 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2590,7 +2590,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2605,34 +2605,34 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2652,39 +2652,39 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2694,17 +2694,17 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2731,12 +2731,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2746,19 +2746,19 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2778,29 +2778,29 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2815,22 +2815,22 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2857,34 +2857,34 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2909,24 +2909,24 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2941,86 +2941,86 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3052,17 +3052,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -3082,91 +3082,91 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3178,37 +3178,37 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3220,121 +3220,121 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3346,37 +3346,37 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3393,32 +3393,32 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3455,12 +3455,12 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3576,17 +3576,17 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3640,37 +3640,37 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3682,101 +3682,101 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3786,17 +3786,17 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3813,12 +3813,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3833,12 +3833,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3850,42 +3850,126 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G82" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr">
+      <c r="H84" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H82"/>
+  <autoFilter ref="A1:H84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-28 19:57 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -915,12 +915,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -999,12 +999,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1014,17 +1014,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Publicação de Editais de Alienação de Imóveis</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1377,32 +1377,32 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
@@ -1419,32 +1419,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1938,17 +1938,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2368,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3393,32 +3393,32 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3445,22 +3445,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3487,22 +3487,22 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3571,22 +3571,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3687,32 +3687,32 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-29 18:25 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -915,12 +915,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -930,17 +930,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Publicação de Editais de Alienação de Imóveis</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -957,12 +957,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -977,12 +977,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1014,17 +1014,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1377,32 +1377,32 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1419,32 +1419,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1938,17 +1938,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2368,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3393,32 +3393,32 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3445,22 +3445,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3487,22 +3487,22 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3571,22 +3571,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3687,32 +3687,32 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-09-30 18:14 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -930,17 +930,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -957,12 +957,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Publicação de Editais de Alienação de Imóveis</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -999,12 +999,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1377,32 +1377,32 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
@@ -1419,32 +1419,32 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1896,17 +1896,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1938,17 +1938,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2368,7 +2368,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3393,32 +3393,32 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3445,22 +3445,22 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3487,22 +3487,22 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3529,22 +3529,22 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3571,22 +3571,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3687,32 +3687,32 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-04 17:14 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$88</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,106 +485,106 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-27T17:23:55</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-22T00:00:00</t>
+          <t>2026-10-01T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
+          <t>Alteração na Diretoria</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1573399&amp;numSequencia=1098105&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-27T17:23:55</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-21T00:00:00</t>
+          <t>2026-09-30T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572717&amp;numSequencia=1097423&amp;numVersao=6</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-18T00:00:00</t>
+          <t>2026-09-29T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -599,24 +599,24 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
+          <t>Corretora GPA</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572643&amp;numSequencia=1097349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-28T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -631,34 +631,34 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Informações Adicionais referentes às Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572221&amp;numSequencia=1096927&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-22T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -673,64 +673,64 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-21T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-18T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -757,22 +757,22 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -925,22 +925,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -994,17 +994,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1019,12 +1019,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Publicação de Editais de Alienação de Imóveis</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1036,101 +1036,101 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-15T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Reenquadramento da cotação das ações da Companhia</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-11T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-10T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1145,24 +1145,24 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Alteração de Membros do Conselho de Administração</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-09T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1187,222 +1187,222 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-08T00:00:00</t>
+          <t>2026-09-15T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Reenquadramento da cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-11T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-10T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Alteração de Membros do Conselho de Administração</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-09T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-08T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1439,12 +1439,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1456,37 +1456,37 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1498,91 +1498,91 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-24T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1597,34 +1597,34 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1639,44 +1639,44 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-18T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1708,17 +1708,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1728,17 +1728,17 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1750,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1770,81 +1770,81 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1854,39 +1854,39 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1901,34 +1901,34 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1938,17 +1938,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1960,37 +1960,37 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2002,37 +2002,37 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2044,17 +2044,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2064,17 +2064,17 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2101,160 +2101,160 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2269,34 +2269,34 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2311,64 +2311,64 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2395,160 +2395,160 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2573,66 +2573,66 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2652,81 +2652,81 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2736,71 +2736,71 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2815,44 +2815,44 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2862,29 +2862,29 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2899,34 +2899,34 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2941,34 +2941,34 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2983,34 +2983,34 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3030,249 +3030,249 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3287,24 +3287,24 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3324,113 +3324,113 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3445,44 +3445,44 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3497,12 +3497,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3514,37 +3514,37 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3571,22 +3571,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3670,7 +3670,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3687,32 +3687,32 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3724,37 +3724,37 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3766,17 +3766,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3791,24 +3791,24 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3823,34 +3823,34 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
-        </is>
-      </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3865,111 +3865,279 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G88" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="H88" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H84"/>
+  <autoFilter ref="A1:H88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-05 21:00 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -809,12 +809,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3571,22 +3571,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3687,32 +3687,32 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3749,12 +3749,12 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3771,32 +3771,32 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3823,22 +3823,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-06 18:44 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -809,12 +809,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3581,12 +3581,12 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3687,32 +3687,32 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3729,32 +3729,32 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3823,22 +3823,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-07 19:10 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -809,12 +809,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3561,32 +3561,32 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3613,22 +3613,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3697,22 +3697,22 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3729,32 +3729,32 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3823,22 +3823,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3875,12 +3875,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-08 19:06 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -809,12 +809,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3561,32 +3561,32 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3623,12 +3623,12 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3697,22 +3697,22 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3739,22 +3739,22 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3823,22 +3823,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3855,32 +3855,32 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-09 18:37 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -809,12 +809,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3571,22 +3571,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3603,32 +3603,32 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3655,22 +3655,22 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3697,22 +3697,22 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3739,22 +3739,22 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3833,12 +3833,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3855,32 +3855,32 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-10 17:35 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -809,12 +809,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -841,22 +841,22 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -888,17 +888,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3571,22 +3571,22 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3603,32 +3603,32 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3665,12 +3665,12 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3697,22 +3697,22 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3739,22 +3739,22 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3813,32 +3813,32 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-11 17:52 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,22 +485,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01T00:00:00</t>
+          <t>2026-10-08T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -515,39 +515,39 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Alteração na Diretoria</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1573399&amp;numSequencia=1098105&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575329&amp;numSequencia=1100035&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-30T00:00:00</t>
+          <t>2026-10-07T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -557,34 +557,34 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572717&amp;numSequencia=1097423&amp;numVersao=6</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-29T00:00:00</t>
+          <t>2026-10-07T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -594,39 +594,39 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Corretora GPA</t>
+          <t>Esclarecimento sobre noticia vinculada na mídia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572643&amp;numSequencia=1097349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575274&amp;numSequencia=1099980&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-28T00:00:00</t>
+          <t>2026-10-07T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -641,24 +641,24 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Informações Adicionais referentes às Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572221&amp;numSequencia=1096927&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-27T17:23:55</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-22T00:00:00</t>
+          <t>2026-10-05T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -673,160 +673,160 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGESP</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
+          <t>(i) a sustação dos efeitos do Evento de Inadimplemento Automático previsto na cláusula 6.1, (vi) do Termo de Emissão||(ii) a aprovação da incorporação dos juros apurados até o dia 25 de setembro de 2026 (inclusive), ao Valor Nominal Unitário das Notas Comerciais Escriturais||(iii) a alteração das Datas de Pagamento da Remuneração das Notas Comerciais Escriturais||(iv) caso aprovadas as matérias previstas nos itens anteriores, alteração das Cláusulas 4.2.2.1, 4.2.2.2 e 4.3.1 do Termo de Emissão, de forma a refletir a incorporação dos juros e o novo cronograma d||(v) autorização para a Emitente e para o Agente Fiduciário adotarem todas as medidas necessárias para refletir e formalizar a efetivação das deliberações constantes na Ordem do Dia</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574085&amp;numSequencia=1098791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-27T17:23:55</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-21T00:00:00</t>
+          <t>2026-10-01T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
+          <t>Alteração na Diretoria</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1573399&amp;numSequencia=1098105&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-18T00:00:00</t>
+          <t>2026-09-30T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572717&amp;numSequencia=1097423&amp;numVersao=6</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-29T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Corretora GPA</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572643&amp;numSequencia=1097349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-28T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -841,34 +841,34 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Informações Adicionais referentes às Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572221&amp;numSequencia=1096927&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-22T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -883,64 +883,64 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-21T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -952,7 +952,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-18T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -967,22 +967,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1009,22 +1009,22 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1061,12 +1061,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1093,22 +1093,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1120,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1135,22 +1135,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1162,37 +1162,37 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Publicação de Editais de Alienação de Imóveis</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1204,101 +1204,101 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-15T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Reenquadramento da cotação das ações da Companhia</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-11T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-10T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1313,34 +1313,34 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Alteração de Membros do Conselho de Administração</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-09T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1350,39 +1350,39 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-08T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1392,227 +1392,227 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-15T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Reenquadramento da cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-11T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-10T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração de Membros do Conselho de Administração</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-09T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-08T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1624,37 +1624,37 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1666,133 +1666,133 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-08-24T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1807,44 +1807,44 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-18T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1859,24 +1859,24 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1891,22 +1891,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1918,17 +1918,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1938,29 +1938,29 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1980,81 +1980,81 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2064,39 +2064,39 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2106,59 +2106,59 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2185,22 +2185,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2212,17 +2212,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2237,12 +2237,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2254,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2269,34 +2269,34 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2316,29 +2316,29 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2353,54 +2353,54 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2410,61 +2410,61 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2479,34 +2479,34 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2521,44 +2521,44 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2568,155 +2568,155 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2731,34 +2731,34 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2773,44 +2773,44 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2825,66 +2825,66 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2904,113 +2904,113 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3030,71 +3030,71 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3109,34 +3109,34 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3151,34 +3151,34 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3203,34 +3203,34 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3240,207 +3240,207 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -3450,39 +3450,39 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3492,123 +3492,123 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3623,24 +3623,24 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3655,44 +3655,44 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -3707,12 +3707,12 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3724,37 +3724,37 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3813,32 +3813,32 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3855,32 +3855,32 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3892,37 +3892,37 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3934,17 +3934,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3959,24 +3959,24 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3991,34 +3991,34 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4038,106 +4038,316 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>Deferimento RJ</t>
-        </is>
-      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G88" t="inlineStr">
+      <c r="G93" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="H93" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H88"/>
+  <autoFilter ref="A1:H93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-12 21:30 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2437,22 +2437,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2847,32 +2847,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2889,32 +2889,32 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3833,12 +3833,12 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3855,12 +3855,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3870,17 +3870,17 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3907,22 +3907,22 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3949,22 +3949,22 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3981,32 +3981,32 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4075,22 +4075,22 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-13 19:42 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2437,22 +2437,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2847,32 +2847,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2889,32 +2889,32 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3823,22 +3823,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3897,32 +3897,32 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3949,22 +3949,22 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3981,12 +3981,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3996,17 +3996,17 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4043,12 +4043,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4075,22 +4075,22 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-14 17:44 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2437,22 +2437,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2847,32 +2847,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2889,32 +2889,32 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3823,22 +3823,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3875,12 +3875,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3897,12 +3897,12 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3912,17 +3912,17 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3939,32 +3939,32 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3991,22 +3991,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4075,22 +4075,22 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-15 17:32 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2437,22 +2437,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2847,32 +2847,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2889,32 +2889,32 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3771,32 +3771,32 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3823,22 +3823,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3907,22 +3907,22 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3939,12 +3939,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3954,17 +3954,17 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4001,12 +4001,12 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4075,22 +4075,22 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-16 17:08 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2437,22 +2437,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2847,32 +2847,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2889,32 +2889,32 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3771,12 +3771,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -3786,17 +3786,17 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3823,22 +3823,22 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3917,12 +3917,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3949,22 +3949,22 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3991,22 +3991,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4065,32 +4065,32 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-17 16:04 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2395,22 +2395,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2437,22 +2437,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2847,32 +2847,32 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2889,32 +2889,32 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3781,22 +3781,22 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3813,32 +3813,32 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3907,22 +3907,22 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3959,12 +3959,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3991,22 +3991,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4065,12 +4065,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4080,17 +4080,17 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-18 16:19 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:H95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,84 +485,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-11T17:52:27</t>
+          <t>2026-10-18T16:19:09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-08T00:00:00</t>
+          <t>2026-10-17T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575329&amp;numSequencia=1100035&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578120&amp;numSequencia=1102826&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-11T17:52:27</t>
+          <t>2026-10-18T16:19:09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-07T00:00:00</t>
+          <t>2026-10-14T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Homologação Plano de Recuperação Extrajudicial</t>
+          <t>Resultado dos Processos Competitivos de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1577239&amp;numSequencia=1101945&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -574,37 +574,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-07T00:00:00</t>
+          <t>2026-10-08T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Esclarecimento sobre noticia vinculada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575274&amp;numSequencia=1099980&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575329&amp;numSequencia=1100035&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-05T00:00:00</t>
+          <t>2026-10-07T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -673,44 +673,44 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AGESP</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>(i) a sustação dos efeitos do Evento de Inadimplemento Automático previsto na cláusula 6.1, (vi) do Termo de Emissão||(ii) a aprovação da incorporação dos juros apurados até o dia 25 de setembro de 2026 (inclusive), ao Valor Nominal Unitário das Notas Comerciais Escriturais||(iii) a alteração das Datas de Pagamento da Remuneração das Notas Comerciais Escriturais||(iv) caso aprovadas as matérias previstas nos itens anteriores, alteração das Cláusulas 4.2.2.1, 4.2.2.2 e 4.3.1 do Termo de Emissão, de forma a refletir a incorporação dos juros e o novo cronograma d||(v) autorização para a Emitente e para o Agente Fiduciário adotarem todas as medidas necessárias para refletir e formalizar a efetivação das deliberações constantes na Ordem do Dia</t>
+          <t>Esclarecimento sobre noticia vinculada na mídia</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574085&amp;numSequencia=1098791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575274&amp;numSequencia=1099980&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-01T00:00:00</t>
+          <t>2026-10-07T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -725,54 +725,54 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Alteração na Diretoria</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1573399&amp;numSequencia=1098105&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-30T00:00:00</t>
+          <t>2026-10-05T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGESP</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>(i) a sustação dos efeitos do Evento de Inadimplemento Automático previsto na cláusula 6.1, (vi) do Termo de Emissão||(ii) a aprovação da incorporação dos juros apurados até o dia 25 de setembro de 2026 (inclusive), ao Valor Nominal Unitário das Notas Comerciais Escriturais||(iii) a alteração das Datas de Pagamento da Remuneração das Notas Comerciais Escriturais||(iv) caso aprovadas as matérias previstas nos itens anteriores, alteração das Cláusulas 4.2.2.1, 4.2.2.2 e 4.3.1 do Termo de Emissão, de forma a refletir a incorporação dos juros e o novo cronograma d||(v) autorização para a Emitente e para o Agente Fiduciário adotarem todas as medidas necessárias para refletir e formalizar a efetivação das deliberações constantes na Ordem do Dia</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572717&amp;numSequencia=1097423&amp;numVersao=6</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574085&amp;numSequencia=1098791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -784,37 +784,37 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-29T00:00:00</t>
+          <t>2026-10-01T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Corretora GPA</t>
+          <t>Alteração na Diretoria</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572643&amp;numSequencia=1097349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1573399&amp;numSequencia=1098105&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -826,59 +826,59 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-28T00:00:00</t>
+          <t>2026-09-30T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Informações Adicionais referentes às Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572221&amp;numSequencia=1096927&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572717&amp;numSequencia=1097423&amp;numVersao=6</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-27T17:23:55</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-22T00:00:00</t>
+          <t>2026-09-29T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -893,34 +893,34 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
+          <t>Corretora GPA</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572643&amp;numSequencia=1097349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-27T17:23:55</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-21T00:00:00</t>
+          <t>2026-09-28T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -935,24 +935,24 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
+          <t>Informações Adicionais referentes às Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572221&amp;numSequencia=1096927&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-18T00:00:00</t>
+          <t>2026-09-22T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -982,49 +982,49 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-21T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-18T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1051,22 +1051,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1098,17 +1098,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1140,17 +1140,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1177,22 +1177,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1219,22 +1219,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1266,17 +1266,17 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1330,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1345,22 +1345,22 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1377,12 +1377,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1392,17 +1392,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Publicação de Editais de Alienação de Imóveis</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1414,121 +1414,121 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-15T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Reenquadramento da cotação das ações da Companhia</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-11T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-10T00:00:00</t>
+          <t>2026-09-15T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Alteração de Membros do Conselho de Administração</t>
+          <t>Reenquadramento da cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1540,37 +1540,37 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-09T00:00:00</t>
+          <t>2026-09-11T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
+          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1582,17 +1582,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-08T00:00:00</t>
+          <t>2026-09-10T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1602,29 +1602,29 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Alteração de Membros do Conselho de Administração</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-09T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1639,64 +1639,64 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-08T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1750,37 +1750,37 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1792,37 +1792,37 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
         </is>
       </c>
     </row>
@@ -1834,37 +1834,37 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1876,22 +1876,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1901,34 +1901,34 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-24T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1943,24 +1943,24 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1975,22 +1975,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2002,37 +2002,37 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-18T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2086,37 +2086,37 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2148,29 +2148,29 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2195,34 +2195,34 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2232,17 +2232,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2254,17 +2254,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2274,17 +2274,17 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2296,17 +2296,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2316,17 +2316,17 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2338,37 +2338,37 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2380,37 +2380,37 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2422,37 +2422,37 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2464,59 +2464,59 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2531,66 +2531,66 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2605,64 +2605,64 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2746,7 +2746,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2773,128 +2773,128 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2904,39 +2904,39 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2946,81 +2946,81 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -3035,12 +3035,12 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3067,34 +3067,34 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3114,59 +3114,59 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3178,7 +3178,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -3198,29 +3198,29 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3240,29 +3240,29 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3277,22 +3277,22 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3319,34 +3319,34 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3371,24 +3371,24 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3403,86 +3403,86 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3497,12 +3497,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3514,17 +3514,17 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3544,19 +3544,19 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3571,64 +3571,64 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3640,37 +3640,37 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3682,121 +3682,121 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3808,37 +3808,37 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3897,32 +3897,32 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3949,12 +3949,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3964,7 +3964,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3991,22 +3991,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4043,12 +4043,12 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4080,17 +4080,17 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4102,17 +4102,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4127,12 +4127,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4144,101 +4144,101 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Alienação de Ativos HNT São Paulo</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-13T00:00:00</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4248,17 +4248,17 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Apresentação de Resultado 1T26</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4275,12 +4275,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4312,42 +4312,126 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr">
+      <c r="G95" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr">
+      <c r="H95" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H93"/>
+  <autoFilter ref="A1:H95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-19 18:56 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3875,12 +3875,12 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3897,32 +3897,32 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3949,22 +3949,22 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3991,22 +3991,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4075,22 +4075,22 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4107,12 +4107,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4122,17 +4122,17 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-20 17:43 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3939,12 +3939,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3954,17 +3954,17 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3991,22 +3991,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4075,22 +4075,22 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4107,32 +4107,32 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4169,12 +4169,12 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-21 17:49 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3917,12 +3917,12 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3939,32 +3939,32 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3991,22 +3991,22 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4065,12 +4065,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -4080,17 +4080,17 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4132,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4159,22 +4159,22 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-22 17:49 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3907,22 +3907,22 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3981,12 +3981,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3996,17 +3996,17 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4033,22 +4033,22 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4065,32 +4065,32 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4127,12 +4127,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4159,22 +4159,22 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-23 17:39 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -3865,22 +3865,22 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3907,22 +3907,22 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3959,12 +3959,12 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3981,32 +3981,32 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4023,12 +4023,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4038,17 +4038,17 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4090,7 +4090,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4117,22 +4117,22 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4159,22 +4159,22 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-24 16:24 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -2479,22 +2479,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -2521,22 +2521,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3855,12 +3855,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3870,17 +3870,17 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3907,22 +3907,22 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -3949,22 +3949,22 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4023,32 +4023,32 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4085,12 +4085,12 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4117,22 +4117,22 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4159,22 +4159,22 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-25 16:56 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Eventos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Eventos'!$A$1:$H$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H95"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -485,106 +485,106 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-18T16:19:09</t>
+          <t>2026-10-25T16:56:16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-17T00:00:00</t>
+          <t>2026-10-22T00:00:00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Mapa Sintético Consolidado</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578120&amp;numSequencia=1102826&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1579524&amp;numSequencia=1104230&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-18T16:19:09</t>
+          <t>2026-10-25T16:56:16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-14T00:00:00</t>
+          <t>2026-10-21T00:00:00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Resultado dos Processos Competitivos de Alienação de Imóveis</t>
+          <t>Publicac¸a~o da Homologac¸a~o do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1577239&amp;numSequencia=1101945&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578908&amp;numSequencia=1103614&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-11T17:52:27</t>
+          <t>2026-10-25T16:56:16</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-08T00:00:00</t>
+          <t>2026-10-21T00:00:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -599,71 +599,71 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deferimento do pedido de Recuperação Judicial</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575329&amp;numSequencia=1100035&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1579129&amp;numSequencia=1103835&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-11T17:52:27</t>
+          <t>2026-10-25T16:56:16</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-07T00:00:00</t>
+          <t>2026-10-19T00:00:00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
+          <t>Ratificação do Pedido de Recuperação Judicial</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578469&amp;numSequencia=1103175&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-11T17:52:27</t>
+          <t>2026-10-25T16:56:16</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-07T00:00:00</t>
+          <t>2026-10-19T00:00:00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -678,76 +678,76 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Esclarecimento sobre noticia vinculada na mídia</t>
+          <t>Alteração do jornal para publicações legais da Companhia</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575274&amp;numSequencia=1099980&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578470&amp;numSequencia=1103176&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-11T17:52:27</t>
+          <t>2026-10-25T16:56:16</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-07T00:00:00</t>
+          <t>2026-10-19T00:00:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Homologação Plano de Recuperação Extrajudicial</t>
+          <t>Mapa Final Detalhado</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578478&amp;numSequencia=1103184&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-11T17:52:27</t>
+          <t>2026-10-25T16:56:16</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-05T00:00:00</t>
+          <t>2026-10-19T00:00:00</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>GRUPO CASAS BAHIA S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -762,39 +762,39 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AGESP</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>(i) a sustação dos efeitos do Evento de Inadimplemento Automático previsto na cláusula 6.1, (vi) do Termo de Emissão||(ii) a aprovação da incorporação dos juros apurados até o dia 25 de setembro de 2026 (inclusive), ao Valor Nominal Unitário das Notas Comerciais Escriturais||(iii) a alteração das Datas de Pagamento da Remuneração das Notas Comerciais Escriturais||(iv) caso aprovadas as matérias previstas nos itens anteriores, alteração das Cláusulas 4.2.2.1, 4.2.2.2 e 4.3.1 do Termo de Emissão, de forma a refletir a incorporação dos juros e o novo cronograma d||(v) autorização para a Emitente e para o Agente Fiduciário adotarem todas as medidas necessárias para refletir e formalizar a efetivação das deliberações constantes na Ordem do Dia</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias deliberadas||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (iv) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574085&amp;numSequencia=1098791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578471&amp;numSequencia=1103177&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-25T16:56:16</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-01T00:00:00</t>
+          <t>2026-10-19T00:00:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -809,76 +809,76 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Alteração na Diretoria</t>
+          <t>Encerramento da Recuperação Judicial</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1573399&amp;numSequencia=1098105&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578480&amp;numSequencia=1103186&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-18T16:19:09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-30T00:00:00</t>
+          <t>2026-10-17T00:00:00</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572717&amp;numSequencia=1097423&amp;numVersao=6</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1578120&amp;numSequencia=1102826&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-18T16:19:09</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-09-29T00:00:00</t>
+          <t>2026-10-14T00:00:00</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -893,118 +893,118 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Corretora GPA</t>
+          <t>Resultado dos Processos Competitivos de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572643&amp;numSequencia=1097349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1577239&amp;numSequencia=1101945&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-04T17:14:16</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-09-28T00:00:00</t>
+          <t>2026-10-08T00:00:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Informações Adicionais referentes às Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572221&amp;numSequencia=1096927&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575329&amp;numSequencia=1100035&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-27T17:23:55</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-09-22T00:00:00</t>
+          <t>2026-10-07T00:00:00</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-27T17:23:55</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-09-21T00:00:00</t>
+          <t>2026-10-07T00:00:00</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1014,39 +1014,39 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
+          <t>Esclarecimento sobre noticia vinculada na mídia</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575274&amp;numSequencia=1099980&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-18T00:00:00</t>
+          <t>2026-10-07T00:00:00</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1061,24 +1061,24 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-11T17:52:27</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-10-05T00:00:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1098,155 +1098,155 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGESP</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>(i) a sustação dos efeitos do Evento de Inadimplemento Automático previsto na cláusula 6.1, (vi) do Termo de Emissão||(ii) a aprovação da incorporação dos juros apurados até o dia 25 de setembro de 2026 (inclusive), ao Valor Nominal Unitário das Notas Comerciais Escriturais||(iii) a alteração das Datas de Pagamento da Remuneração das Notas Comerciais Escriturais||(iv) caso aprovadas as matérias previstas nos itens anteriores, alteração das Cláusulas 4.2.2.1, 4.2.2.2 e 4.3.1 do Termo de Emissão, de forma a refletir a incorporação dos juros e o novo cronograma d||(v) autorização para a Emitente e para o Agente Fiduciário adotarem todas as medidas necessárias para refletir e formalizar a efetivação das deliberações constantes na Ordem do Dia</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574085&amp;numSequencia=1098791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-10-01T00:00:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Alteração na Diretoria</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1573399&amp;numSequencia=1098105&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-30T00:00:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572717&amp;numSequencia=1097423&amp;numVersao=6</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-29T00:00:00</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Corretora GPA</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572643&amp;numSequencia=1097349&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-10-04T17:14:16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-28T00:00:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1261,34 +1261,34 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Informações Adicionais referentes às Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1572221&amp;numSequencia=1096927&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-22T00:00:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1303,64 +1303,64 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570313&amp;numSequencia=1095019&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-21T18:25:36</t>
+          <t>2026-09-27T17:23:55</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-09-17T00:00:00</t>
+          <t>2026-09-21T00:00:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Fechamento da operação de venda dos ativos da Loja HNT da Vila Mariana</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1570246&amp;numSequencia=1094952&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-18T00:00:00</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1392,17 +1392,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Alteração na composição da Diretoria Estatutária e no Comitê de Auditoria Riscos e Compliance da Companhia</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569617&amp;numSequencia=1094323&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1414,37 +1414,37 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Publicação de Editais de Alienação de Imóveis</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-09-16T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1481,12 +1481,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1498,175 +1498,175 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-09-15T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Reenquadramento da cotação das ações da Companhia</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-09-11T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
-        </is>
-      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569304&amp;numSequencia=1094010&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-09-10T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Alteração de Membros do Conselho de Administração</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-09-09T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-14T18:18:20</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-09-08T00:00:00</t>
+          <t>2026-09-17T00:00:00</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1681,76 +1681,76 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Procedimentos para reenquadramento do Valor Mínimo de Cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568759&amp;numSequencia=1093465&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1765,118 +1765,118 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Publicação de Editais de Alienação de Imóveis</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568911&amp;numSequencia=1093617&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2026-09-03T00:00:00</t>
+          <t>2026-09-16T00:00:00</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568758&amp;numSequencia=1093464&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-21T18:25:36</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-15T00:00:00</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Mapa de Votação Sintético Consolidado AGE</t>
+          <t>Reenquadramento da cotação das ações da Companhia</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1568195&amp;numSequencia=1092901&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2026-09-01T00:00:00</t>
+          <t>2026-09-11T00:00:00</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1901,24 +1901,24 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Tratamento excepcional | Desenquadramento do percentual mínimo de ações em circulação no mercado | Extensão automática de prazo pela B3</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567396&amp;numSequencia=1092102&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-10T00:00:00</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1938,81 +1938,81 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>Alteração de Membros do Conselho de Administração</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1567130&amp;numSequencia=1091836&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-09-06T15:56:33</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2026-08-31T00:00:00</t>
+          <t>2026-09-09T00:00:00</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
+          <t>AMERICANAS Reconhecida como Marca de Alto Renome</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1566430&amp;numSequencia=1091136&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-14T18:18:20</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2026-08-24T00:00:00</t>
+          <t>2026-09-08T00:00:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2027,192 +2027,192 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1565933&amp;numSequencia=1090639&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-08-21T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564397&amp;numSequencia=1089103&amp;numVersao=5</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-08-18T00:00:00</t>
+          <t>2026-09-03T00:00:00</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
+          <t>Mapa de Votação Sintético Consolidado AGE</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563704&amp;numSequencia=1088410&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-08-26T13:50:00</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-08-17T00:00:00</t>
+          <t>2026-09-01T00:00:00</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2227,44 +2227,44 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 2T26</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1563387&amp;numSequencia=1088093&amp;numVersao=4</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-08-16T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2274,81 +2274,81 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 2T26</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562894&amp;numSequencia=1087600&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-09-06T15:56:33</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-08-14T00:00:00</t>
+          <t>2026-08-31T00:00:00</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Disponibilização Term Sheet na CVM</t>
+          <t>Deferimento de Tutela de Urgência na Recuperação Judicial</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1562849&amp;numSequencia=1087555&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-24T00:00:00</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>CVLB BRASIL S.A EM RECUPERAÇÃO JUDICAL</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -2358,39 +2358,39 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
+          <t>Resposta Ofício nº 241/2026-SLE, de 11/08/2026, sobre o andamento do proc. de recuperação judicial e, em especial, da apresentação de objeções ao Plano de Recuperação Judicial.</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560634&amp;numSequencia=1085340&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>2026-08-13T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2400,71 +2400,71 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 2T26</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560487&amp;numSequencia=1085193&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-08-12T00:00:00</t>
+          <t>2026-08-21T00:00:00</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1560332&amp;numSequencia=1085038&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-18T00:00:00</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2479,44 +2479,44 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Calendário de Eventos Corporativos</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Esclarecimentos acerca de notícia veiculada na mídia</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1559232&amp;numSequencia=1083938&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-08-11T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2526,81 +2526,81 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Alteração do Calendário de Eventos Corporativos</t>
+          <t>Apresentação de resultados 2T26</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558416&amp;numSequencia=1083122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-08-16T13:26:02</t>
+          <t>2026-08-26T13:50:00</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-08-10T00:00:00</t>
+          <t>2026-08-17T00:00:00</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>Apresentação de Resultado 2T26 - Videoconferência</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558693&amp;numSequencia=1083399&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-08-07T00:00:00</t>
+          <t>2026-08-16T00:00:00</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2610,29 +2610,29 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
+          <t>Apresentação de Resultado 2T26</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558370&amp;numSequencia=1083076&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-08-09T13:44:03</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-08-04T00:00:00</t>
+          <t>2026-08-14T00:00:00</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2652,29 +2652,29 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 2T26</t>
+          <t>Disponibilização Term Sheet na CVM</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1558099&amp;numSequencia=1082805&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2689,34 +2689,34 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Comunicado ao Mercado - Fechamento Inicial HNT</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1557416&amp;numSequencia=1082122&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-13T00:00:00</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2731,128 +2731,128 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>Apresentação de Resultados 2T26</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556826&amp;numSequencia=1081532&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-12T00:00:00</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Term Sheet das debêntures do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556765&amp;numSequencia=1081471&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>2026-07-30T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556064&amp;numSequencia=1080770&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-08-02T14:25:34</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>2026-07-27T00:00:00</t>
+          <t>2026-08-11T00:00:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2867,76 +2867,76 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>CAM 236 23 Instauração da arbitragem</t>
+          <t>Alteração do Calendário de Eventos Corporativos</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1556065&amp;numSequencia=1080771&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-07-26T14:26:00</t>
+          <t>2026-08-16T13:26:02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>2026-07-20T00:00:00</t>
+          <t>2026-08-10T00:00:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Alteração na Administração da Companhia</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1555456&amp;numSequencia=1080162&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-08-07T00:00:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2946,71 +2946,71 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Notícia Veiculada na Mídia</t>
+          <t>Conclusão do procedimento de ajuste de preço da alienação da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1554573&amp;numSequencia=1079279&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-20T15:06:32</t>
+          <t>2026-08-09T13:44:03</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>2026-07-17T00:00:00</t>
+          <t>2026-08-04T00:00:00</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Aumento do capital social da Companhia</t>
+          <t>Apresentação de Resultado - 2T26</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1552160&amp;numSequencia=1076866&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-07-13T15:39:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>2026-07-09T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -3025,34 +3025,34 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550028&amp;numSequencia=1074734&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2026-07-03T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -3067,76 +3067,76 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
+          <t>AGE</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
           <t>nan</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>Conclusão da Venda da UPI Uni.Co</t>
-        </is>
-      </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550029&amp;numSequencia=1074735&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>2026-07-02T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Conclusão Operação Stix</t>
+          <t>Autorizar a alteração do caput do Artigo 5º do Estatuto Social da Companhia para refletir o novo valor e o número de ações, consolidar o Estatuto Social da Companhia de forma a refletir as alterações,</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550023&amp;numSequencia=1074729&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-07-06T16:16:07</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>2026-06-30T00:00:00</t>
+          <t>2026-07-30T00:00:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3151,44 +3151,44 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Notícia divulgada na mídia</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1550030&amp;numSequencia=1074736&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-08-02T14:25:34</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>2026-06-26T00:00:00</t>
+          <t>2026-07-27T00:00:00</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -3198,39 +3198,39 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>CAM 236 23 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1548063&amp;numSequencia=1072769&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-26T14:26:00</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-20T00:00:00</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -3245,34 +3245,34 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Eleição DRI</t>
+          <t>Alteração na Administração da Companhia</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546409&amp;numSequencia=1071115&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-06-28T14:45:29</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>2026-06-22T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -3282,29 +3282,29 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Aumento do capital social da Companhia</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546085&amp;numSequencia=1070791&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-20T15:06:32</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2026-06-17T00:00:00</t>
+          <t>2026-07-17T00:00:00</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3324,113 +3324,113 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Notícia Veiculada na Mídia</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1546074&amp;numSequencia=1070780&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-13T15:39:29</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2026-06-16T00:00:00</t>
+          <t>2026-07-09T00:00:00</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
+          <t>Esclarecimentos Sobre a Recuperação Judicial</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1543326&amp;numSequencia=1068032&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-21T15:09:12</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2026-06-15T00:00:00</t>
+          <t>2026-07-03T00:00:00</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Ata</t>
+          <t>Conclusão da Venda da UPI Uni.Co</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541658&amp;numSequencia=1066364&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>2026-06-13T00:00:00</t>
+          <t>2026-07-02T00:00:00</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3445,44 +3445,44 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
+          <t>Conclusão Operação Stix</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1541402&amp;numSequencia=1066108&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-15T17:59:57</t>
+          <t>2026-07-06T16:16:07</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>2026-06-10T00:00:00</t>
+          <t>2026-06-30T00:00:00</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3492,39 +3492,39 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
+          <t>Notícia divulgada na mídia</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1540179&amp;numSequencia=1064885&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2026-05-29T00:00:00</t>
+          <t>2026-06-26T00:00:00</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3534,81 +3534,81 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1538953&amp;numSequencia=1063659&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>2026-05-27T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>CAM 294 25 Instauração da arbitragem</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537044&amp;numSequencia=1061750&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-05-31T14:28:17</t>
+          <t>2026-06-28T14:45:29</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>2026-05-26T00:00:00</t>
+          <t>2026-06-22T00:00:00</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3618,113 +3618,113 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Mudança na composição do comitê de auditoria estatutário</t>
+          <t>Eleição DRI</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1537040&amp;numSequencia=1061746&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-17T00:00:00</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Aquisição/Alienação de Participação Acionária (art. 12 da Instr. CVM nº 358)</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Reforma Estatutária</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1535700&amp;numSequencia=1060406&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>2026-05-22T00:00:00</t>
+          <t>2026-06-16T00:00:00</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Outros avisos</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Aumento de capital por exercício de bônus de subscrição</t>
+          <t>AGE 15/06 - Mapa Final de Votação Detalhado</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534915&amp;numSequencia=1059621&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-21T15:09:12</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>2026-05-20T00:00:00</t>
+          <t>2026-06-15T00:00:00</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3739,128 +3739,128 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Venda da Participação Societária na Stix</t>
+          <t>AGE 15/06 - Ata</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534453&amp;numSequencia=1059159&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-05-24T14:22:09</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>2026-05-18T00:00:00</t>
+          <t>2026-06-13T00:00:00</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>MARISA LOJAS SA</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>61189288000189</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Apresentação de resultados 1T26</t>
+          <t>AGE 15/06 - Mapa Sintético Consolidado</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1534342&amp;numSequencia=1059048&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-06-15T17:59:57</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>2026-05-15T00:00:00</t>
+          <t>2026-06-10T00:00:00</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Alteração Estatuto Social</t>
+          <t>Publicação do Edital do Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1533050&amp;numSequencia=1057756&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-29T00:00:00</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>GRUPO CASAS BAHIA S.A.</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>33041260065290</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -3870,165 +3870,165 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1528651&amp;numSequencia=1053357&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-27T00:00:00</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>CAM 294 25 Instauração da arbitragem</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1527543&amp;numSequencia=1052249&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-31T14:28:17</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-26T00:00:00</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Instalação, mudança ou dissolução do Comitê de Auditoria Estatutário</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Mudança na composição do comitê de auditoria estatutário</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526934&amp;numSequencia=1051640&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros avisos</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Aumento de capital por exercício de bônus de subscrição</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1526422&amp;numSequencia=1051128&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-22T00:00:00</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -4043,24 +4043,24 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Reforma Estatutária</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525884&amp;numSequencia=1050590&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-20T00:00:00</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4075,44 +4075,44 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Venda da Participação Societária na Stix</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1525258&amp;numSequencia=1049964&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-05-17T14:24:03</t>
+          <t>2026-05-24T14:22:09</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-18T00:00:00</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>MARISA LOJAS SA</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>61189288000189</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -4127,12 +4127,12 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de resultados 1T26</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1523458&amp;numSequencia=1048164&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4144,37 +4144,37 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>2026-05-14T00:00:00</t>
+          <t>2026-05-15T00:00:00</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>CVLB BRASIL S.A.</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>16233389000155</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>Alteração Estatuto Social</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522972&amp;numSequencia=1047678&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4186,37 +4186,37 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Alienação de Ativos HNT São Paulo</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4228,17 +4228,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-05-13T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>GRUPO CASAS BAHIA S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>33041260065290</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4248,29 +4248,29 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4285,34 +4285,34 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4327,111 +4327,447 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Notícia veiculada na mídia</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-05-13T19:28:37</t>
+          <t>2026-05-17T14:24:03</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-05-05T00:00:00</t>
+          <t>2026-05-14T00:00:00</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>CVLB BRASIL S.A.</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>16233389000155</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Deferimento RJ</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Convocação AGE</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultados 1T26</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>2026-05-14T00:00:00</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Aviso aos Acionistas</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>GRUPO CASAS BAHIA S.A.</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>33041260065290</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Apresentações a analistas/agentes do mercado</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Apresentação de Resultado 1T26</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521723&amp;numSequencia=1046429&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-05-17T14:24:03</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>2026-05-13T00:00:00</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>00776574000156</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Alienação de Ativos HNT São Paulo</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521643&amp;numSequencia=1046349&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
           <t>2026-05-13T19:28:37</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Celebração de nova versão do plano de recuperação extrajudicial</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516383&amp;numSequencia=1041089&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>47508411000156</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Esclarecimentos sobre questionamentos da CVM/B3</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Notícia veiculada na mídia</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516385&amp;numSequencia=1041091&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>2026-05-05T00:00:00</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>CVLB BRASIL S.A.</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>16233389000155</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Fato Relevante</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Deferimento RJ</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1516335&amp;numSequencia=1041041&amp;numVersao=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-05-13T19:28:37</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
         <is>
           <t>2026-05-04T00:00:00</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D103" t="inlineStr">
         <is>
           <t>00776574000156</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>Comunicado ao Mercado</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Comunicado ao Mercado</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
         <is>
           <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
-      <c r="G95" t="inlineStr">
+      <c r="G103" t="inlineStr">
         <is>
           <t>CAM 268 24 - Desistência dos requerentes</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr">
+      <c r="H103" t="inlineStr">
         <is>
           <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1515450&amp;numSequencia=1040156&amp;numVersao=1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H95"/>
+  <autoFilter ref="A1:H103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-26 18:59 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -957,32 +957,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Homologação Plano de Recuperação Extrajudicial</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1518,17 +1518,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4211,12 +4211,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4243,22 +4243,22 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4275,12 +4275,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4295,12 +4295,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4327,22 +4327,22 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4369,22 +4369,22 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4411,22 +4411,22 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4443,12 +4443,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4458,17 +4458,17 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4495,12 +4495,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-27 18:30 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -957,32 +957,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Homologação Plano de Recuperação Extrajudicial</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1518,17 +1518,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4201,22 +4201,22 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4243,12 +4243,12 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -4258,7 +4258,7 @@
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4275,12 +4275,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -4290,17 +4290,17 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4327,22 +4327,22 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4359,12 +4359,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4379,12 +4379,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4411,22 +4411,22 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4453,22 +4453,22 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4505,12 +4505,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-28 18:36 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -957,32 +957,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Homologação Plano de Recuperação Extrajudicial</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1518,17 +1518,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4191,12 +4191,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4211,12 +4211,12 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4253,12 +4253,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4285,22 +4285,22 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4327,22 +4327,22 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4359,12 +4359,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -4374,17 +4374,17 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4411,22 +4411,22 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4453,12 +4453,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -4468,7 +4468,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4495,22 +4495,22 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-29 18:45 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -957,32 +957,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Homologação Plano de Recuperação Extrajudicial</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1518,17 +1518,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4191,12 +4191,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -4206,17 +4206,17 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4243,22 +4243,22 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4285,12 +4285,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -4300,7 +4300,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4327,22 +4327,22 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4369,22 +4369,22 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4411,22 +4411,22 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4463,12 +4463,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4485,12 +4485,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4505,12 +4505,12 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-30 18:22 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -957,32 +957,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Homologação Plano de Recuperação Extrajudicial</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1518,17 +1518,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4201,22 +4201,22 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4233,12 +4233,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4253,12 +4253,12 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4295,12 +4295,12 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4327,22 +4327,22 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4369,12 +4369,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -4384,7 +4384,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4411,22 +4411,22 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4453,22 +4453,22 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4485,12 +4485,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -4500,17 +4500,17 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza historico e state 2026-10-31 17:28 UTC
</commit_message>
<xml_diff>
--- a/02. Histórico/github-cvm-fatos-relevantes.xlsx
+++ b/02. Histórico/github-cvm-fatos-relevantes.xlsx
@@ -957,32 +957,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
+          <t>Homologação Plano de Recuperação Extrajudicial</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1041,32 +1041,32 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Homologação Plano de Recuperação Extrajudicial</t>
+          <t>Atualização sobre a Venda de Ativos - Lojas Hortifruti Natural da Terra</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1574980&amp;numSequencia=1099686&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1575180&amp;numSequencia=1099886&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1439,12 +1439,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1471,22 +1471,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
+          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1518,17 +1518,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
+          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1602,17 +1602,17 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AGDEB</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Ata da Assembleia Geral de Debenturistas da 11ª emissão de debentures</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Companhia e das demais matérias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Companhia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstraçõe||Ratificar o pedido de Recuperação Judicial da Companhia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569126&amp;numSequencia=1093832&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569301&amp;numSequencia=1094007&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1639,22 +1639,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>AGDEB</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Emissões de Notas Comerciais Escriturais para Colocação Privada</t>
+          <t>Termo de não instalação da Assembleia Geral de Debenturistas da 10ª emissão de debentures</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569306&amp;numSequencia=1094012&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569125&amp;numSequencia=1093831&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -1691,12 +1691,12 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Alterar o caput do artigo 5º do Estatuto Social da Companhia para refletir o aumento de capital da Companhia aprovado em reunião do Conselho de Administração realizada em 16 de julho de 2026||Autorizar os Administradores da Companhia a praticar todos os atos necessários para dar continuidade e garantir a efetivação da recuperação judicial da Cia e demais materias||Consolidar o Estatuto Social da Companhia, de forma a refletir a alteração indicada no item (4) acima||Eleger 1 (um) novo membro efetivo do Conselho Fiscal da Companhia e seu respectivo suplente||Ratificar o número de membros que compõem o Conselho de Administração da Cia para o mandato que se encerrará com a realização da Assembleia Geral Ordinária que deliberará acerca das demonstrações fin||Ratificar o pedido de Recuperação Judicial da Cia, em conjunto com determinadas de suas subsidiárias, ajuizado no dia 16 de agosto de 2026, perante o Juízo de Falências e Recuperações Judiciais</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569302&amp;numSequencia=1094008&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1569303&amp;numSequencia=1094009&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2069,12 +2069,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
+          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -2153,12 +2153,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Alterar, consolidar o Estatuto Social, atualizar o capital social decorrente do exercício de bônus de subscrição, fixar o número, eleger os membros do Conselho de Administração e autorizar...</t>
+          <t>Mapa Final de Votação Detalhado - AGE 03/09/2026</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564717&amp;numSequencia=1089423&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1564715&amp;numSequencia=1089421&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4201,12 +4201,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Aviso aos Acionistas</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -4216,7 +4216,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4233,12 +4233,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
+          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>00776574000156</t>
+          <t>47508411000156</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -4248,17 +4248,17 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Apresentações a analistas/agentes do mercado</t>
+          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Apresentação de Resultados 1T26</t>
+          <t>Renúncia de suplente do Conselho Fiscal</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4285,22 +4285,22 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Comunicado ao Mercado</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>Apresentações a analistas/agentes do mercado</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Apresentação de Resultado - 1T26</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4327,22 +4327,22 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Fato Relevante</t>
+          <t>Assembleia</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AGE</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Convocação AGE</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
         </is>
       </c>
     </row>
@@ -4379,12 +4379,12 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522528&amp;numSequencia=1047234&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522550&amp;numSequencia=1047256&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4411,22 +4411,22 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Assembleia</t>
+          <t>Fato Relevante</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>AGE</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Deliberar sobre alteração de limite do capital autorizado, exclusão do capitulo X do estatuto social dentre outras deliberações</t>
+          <t>Convocação AGE</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522553&amp;numSequencia=1047259&amp;numVersao=2</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522562&amp;numSequencia=1047268&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4443,12 +4443,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>COMPANHIA BRASILEIRA DE DISTRIBUIÇÃO</t>
+          <t>AMERICANAS S.A. - EM RECUPERAÇÃO JUDICIAL</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>47508411000156</t>
+          <t>00776574000156</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4463,12 +4463,12 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Apresentação de Resultado - 1T26</t>
+          <t>Apresentação de Resultados 1T26</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522493&amp;numSequencia=1047199&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1521815&amp;numSequencia=1046521&amp;numVersao=1</t>
         </is>
       </c>
     </row>
@@ -4495,22 +4495,22 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Comunicado ao Mercado</t>
+          <t>Aviso aos Acionistas</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Outros Comunicados Não Considerados Fatos Relevantes</t>
+          <t>Aumento de capital por subscrição privada deliberado em RCA</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Renúncia de suplente do Conselho Fiscal</t>
+          <t>nan</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
         <is>
-          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522503&amp;numSequencia=1047209&amp;numVersao=1</t>
+          <t>https://www.rad.cvm.gov.br/ENET/frmDownloadDocumento.aspx?Tela=ext&amp;descTipo=IPE&amp;CodigoInstituicao=1&amp;numProtocolo=1522515&amp;numSequencia=1047221&amp;numVersao=1</t>
         </is>
       </c>
     </row>

</xml_diff>